<commit_message>
Implemented async successfully with a semaphore of 50, to be able to run multiple PING processes simultaneously, and make the script 10 times faster!
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F6" s="5" t="n"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F18" s="5" t="n"/>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F19" s="5" t="n"/>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F24" s="8" t="n"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F27" s="11" t="n"/>
@@ -1616,7 +1616,7 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>LKBD-BL0006-FL02-RM224-LXMCX942</t>
+          <t>LKBD-BL0006-FL01-RM224-LXMCX942</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F28" s="14" t="n"/>
@@ -1644,7 +1644,7 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>LKBD-BL0006-FL03-RM25-LXMCX942</t>
+          <t>LKBD-BL0006-FL02-RM25-LXMCX942</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F29" s="14" t="n"/>
@@ -1672,7 +1672,7 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>LKBD-BL0006-FL02-RM08-LXMCX942</t>
+          <t>LKBD-BL0006-FL01-RM08-LXMCX942</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
@@ -1692,7 +1692,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -1700,7 +1700,7 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>LKBD-BL0006-FL01-RM01-LXMCX942</t>
+          <t>LKBD-BL0006-GF-RM01-LXMCX942</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F31" s="14" t="n"/>
@@ -1728,7 +1728,7 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>LKBD-BL0006-FL03-RM08-Lexmark921</t>
+          <t>LKBD-BL0006-FL02-RM08-Lexmark921</t>
         </is>
       </c>
       <c r="B32" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Fully Operational: async working as expected, fixed bug that caused async to not repsect the order of status by order of rows in table. The solution was to use async.gather(). Also, fixed details like the title of the report to start with the EXCEL sheet name, ...
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F6" s="5" t="n"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F18" s="5" t="n"/>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="F19" s="5" t="n"/>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F24" s="8" t="n"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F27" s="11" t="n"/>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F28" s="14" t="n"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F29" s="14" t="n"/>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F30" s="14" t="n"/>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F31" s="14" t="n"/>

</xml_diff>

<commit_message>
Fully Operational: added automatic close of EXCEL if open when starting the script, also automatic open of EXCEL and HTML Report at the end, and updated banner and text logs. This new fucntionalities are defined on fucntions in the correspondednt modules.
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -233,7 +233,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill>
@@ -326,6 +326,30 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.3999755851924192"/>
+        </patternFill>
+      </fill>
       <border>
         <left style="thin">
           <color auto="1"/>
@@ -512,11 +536,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:F32" headerRowCount="1" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
-  <autoFilter ref="A1:F32"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="Hostname" dataDxfId="10"/>
-    <tableColumn id="2" name="IP Address" dataDxfId="9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G32" headerRowCount="1" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+  <autoFilter ref="A1:G32"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Hostname" dataDxfId="11"/>
+    <tableColumn id="2" name="IP Address" dataDxfId="10"/>
+    <tableColumn id="6" name="MAC Address" dataDxfId="9"/>
     <tableColumn id="3" name="Serial Number" dataDxfId="8"/>
     <tableColumn id="4" name="Configuration" dataDxfId="7"/>
     <tableColumn id="8" name="Status" dataDxfId="6"/>
@@ -815,14 +840,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="33.1796875" customWidth="1" min="1" max="1"/>
-    <col width="14.1796875" customWidth="1" min="2" max="2"/>
-    <col width="15.6328125" customWidth="1" min="3" max="4"/>
-    <col width="12.26953125" customWidth="1" min="5" max="5"/>
-    <col width="76.1796875" customWidth="1" min="6" max="6"/>
+    <col width="14.1796875" customWidth="1" min="2" max="3"/>
+    <col width="15.54296875" customWidth="1" min="4" max="5"/>
+    <col width="12.26953125" customWidth="1" min="6" max="6"/>
+    <col width="76.1796875" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -836,22 +861,27 @@
           <t>IP Address</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>MAC Address</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Serial Number</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Configuration</t>
         </is>
       </c>
-      <c r="E1" s="20" t="inlineStr">
+      <c r="F1" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Special Notes</t>
         </is>
@@ -870,20 +900,25 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
+          <t>788C770938EC</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
           <t>75800HK700944</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="n"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -898,20 +933,25 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
+          <t>788C770938E8</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>75800HK700912</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Undone</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
       <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>The printer has been reconnected to the MCEN network</t>
         </is>
@@ -930,20 +970,25 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>788C7709386C</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>75800HK700954</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>No fiber connectivity at Postal yet</t>
         </is>
@@ -962,20 +1007,25 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>788C770938A8</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>75800HK700902</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -990,20 +1040,25 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
+          <t>788C77093885</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
           <t>75800HK700819</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Offline</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1018,20 +1073,25 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
+          <t>788C7709388D</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
           <t>75800HK700825</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1046,20 +1106,25 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>788C77093887</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
           <t>75800HK700941</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1074,20 +1139,25 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>788C77093818</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>75800HK700786</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1102,20 +1172,25 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>788C77093834</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
           <t>75800HK700831</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Undone</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Building under maintenance</t>
         </is>
@@ -1134,20 +1209,25 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>788C77093874</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
           <t>75800HK700770</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Undone</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Building under maintenance</t>
         </is>
@@ -1166,20 +1246,25 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
+          <t>788C77093819</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
           <t>75800HK700678</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1194,20 +1279,25 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
+          <t>788C770938D9</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
           <t>75800HK700782</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1222,20 +1312,25 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>788C77093833</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
           <t>75800HK700879</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Pending to get the printer's walljack ID for proper configuration of the switcport</t>
         </is>
@@ -1254,20 +1349,25 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
+          <t>788C77093848</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>75800HK700947</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1282,20 +1382,25 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
+          <t>788C7709382B</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
           <t>75800HK700767</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1310,20 +1415,25 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
+          <t>788C770938E0</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
           <t>75800HK700687</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1338,20 +1448,25 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
+          <t>788C77093845</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
           <t>75800HK700699</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1366,20 +1481,25 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
+          <t>788C77093839</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
           <t>75800HK700695</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1394,20 +1514,25 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
+          <t>788C7709D8C7</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
           <t>75800HK700727</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="n"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1422,20 +1547,25 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
+          <t>788C7709380D</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
           <t>75800HK700914</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1450,20 +1580,25 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
+          <t>788C770938E4</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
           <t>75800HK700915</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n"/>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1478,20 +1613,25 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
+          <t>788C770938B9</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
           <t>75800HK700676</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Offline</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>The MAGTF ACE has unplugged the printer</t>
         </is>
@@ -1510,20 +1650,25 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
+          <t>788C77093807</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
           <t>75800HK700746</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="n"/>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1538,20 +1683,25 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
+          <t>788C770938D7</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
           <t>75800HK700693</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1566,24 +1716,25 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
+          <t>788C77093871</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
           <t>75800HK700681</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>Offline</t>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>The MAGTF ACE has unplugged the printer</t>
-        </is>
-      </c>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -1598,20 +1749,25 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
+          <t>788C7709C84E</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
           <t>75800HK700839</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="n"/>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -1626,20 +1782,25 @@
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
+          <t>788C77093875</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
           <t>75800HK700684</t>
         </is>
       </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F28" s="14" t="n"/>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
@@ -1654,20 +1815,25 @@
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
+          <t>788C77094899</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
           <t>75800HK700845</t>
         </is>
       </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="n"/>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -1682,20 +1848,25 @@
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
+          <t>788C7709C821</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
           <t>75800HK700719</t>
         </is>
       </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="n"/>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
@@ -1710,20 +1881,25 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
+          <t>788C7709C8EE</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
           <t>7559030022660</t>
         </is>
       </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F31" s="14" t="n"/>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
@@ -1738,42 +1914,43 @@
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
+          <t>788C7784528A</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
           <t>75800HK700819</t>
         </is>
       </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E32" s="17" t="inlineStr">
-        <is>
-          <t>Offline</t>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>The MAGTF CE has unplugged the printer</t>
-        </is>
-      </c>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:F22">
+  <conditionalFormatting sqref="A2:G22">
     <cfRule type="expression" priority="5" dxfId="4">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23:F26">
+  <conditionalFormatting sqref="A23:G26">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A28:F32">
+  <conditionalFormatting sqref="A28:G32">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>ISODD(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E1048576">
+  <conditionalFormatting sqref="F1:F1048576">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
       <formula>"Offline"</formula>
     </cfRule>
@@ -1785,7 +1962,7 @@
   <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;L&amp;"Calibri"&amp;10 &amp;K000000_x000d_# DISTRIBUTION: DoW COMMUNITY ONLY</oddFooter>
+    <oddFooter>&amp;L&amp;"Calibri"&amp;10 &amp;K000000_x000d_# DISTRIBUTION: DoW COMMUNITY ONLY_x000d_&amp;1#&amp;"Calibri"&amp;10 &amp;K000000 DISTRIBUTION: DoW COMMUNITY ONLY</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Fully Operational: fixed error handling for empty user input and invalid user input. Consolidated both checks in a single function inside the PrinterCheckerApp class. Fixed comments and other miscellaneous staff.
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -915,7 +915,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G2" s="5" t="n"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G6" s="5" t="n"/>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G8" s="5" t="n"/>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G12" s="5" t="n"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G13" s="5" t="n"/>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G15" s="5" t="n"/>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G16" s="5" t="n"/>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G17" s="5" t="n"/>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G18" s="5" t="n"/>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G20" s="5" t="n"/>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G21" s="5" t="n"/>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G22" s="5" t="n"/>

</xml_diff>

<commit_message>
Fully Operational: use absolute path as an argument for the update_tracker_status and creat_printers_dataframe functions on the data_ops module, and argumented the absolute path (excel_file) when calling them on the main_program file.
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -948,7 +948,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="G6" s="5" t="n"/>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G9" s="5" t="n"/>

</xml_diff>

<commit_message>
Fully Operational: implemented logging 99%, corrected a few misplaced logs, set a cammo background color and some graphical beauty, and corrected bug of the counter not resetting to 0% after errors
</commit_message>
<xml_diff>
--- a/Printer_Fleet_Table.xlsx
+++ b/Printer_Fleet_Table.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="30" windowWidth="19420" windowHeight="10160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-38520" yWindow="7275" windowWidth="38640" windowHeight="20910" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MRF-D" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -841,13 +841,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33.1796875" customWidth="1" min="1" max="1"/>
-    <col width="14.1796875" customWidth="1" min="2" max="3"/>
-    <col width="15.54296875" customWidth="1" min="4" max="5"/>
-    <col width="12.26953125" customWidth="1" min="6" max="6"/>
-    <col width="76.1796875" customWidth="1" min="7" max="7"/>
+    <col width="33.140625" customWidth="1" min="1" max="1"/>
+    <col width="14.140625" customWidth="1" min="2" max="3"/>
+    <col width="15.5703125" customWidth="1" min="4" max="5"/>
+    <col width="12.28515625" customWidth="1" min="6" max="6"/>
+    <col width="76.140625" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -890,7 +890,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ROBO-BL0252-FL1-RM001-LXMCX942</t>
+          <t>ROBO-BL0252-FL1-RM003-LXMCX942</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>214.43.185.84</t>
+          <t>214.43.185.75</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>214.43.185.82</t>
+          <t>214.43.185.90</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G6" s="5" t="n"/>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>214.43.185.83</t>
+          <t>214.43.185.88</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G7" s="5" t="n"/>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Offline</t>
         </is>
       </c>
       <c r="G9" s="5" t="n"/>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Offline</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="G18" s="5" t="n"/>

</xml_diff>